<commit_message>
feat: integrate color configuration system with new schema and helper files
</commit_message>
<xml_diff>
--- a/fast_order_catalog.xlsx
+++ b/fast_order_catalog.xlsx
@@ -1478,7 +1478,11 @@
           <t>مشکی</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#000000</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1491,7 +1495,11 @@
           <t>سفید</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>#FFFFFF</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1504,7 +1512,11 @@
           <t>آبی</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>#0000FF</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1517,7 +1529,11 @@
           <t>نارنجی</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>#FFA500</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1530,7 +1546,11 @@
           <t>سبز</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1543,7 +1563,11 @@
           <t>نقره ای</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#C0C0C0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1556,7 +1580,11 @@
           <t>قرمز</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#FF0000</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1569,7 +1597,11 @@
           <t>سبز</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1582,7 +1614,11 @@
           <t>شفاف</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#FFFFFF</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1595,7 +1631,11 @@
           <t>یاسی</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>#C8A2C8</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1608,7 +1648,11 @@
           <t>خاکستری</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>#808080</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1621,7 +1665,11 @@
           <t>طلایی</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>#FFD700</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1634,7 +1682,11 @@
           <t>سفید طلایی</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>#F5E050</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1647,7 +1699,11 @@
           <t>رنگی</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>#808080</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1660,7 +1716,11 @@
           <t>زرد</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>#FFFF00</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1673,7 +1733,11 @@
           <t>صورتی</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>#FFC0CB</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1686,7 +1750,11 @@
           <t>کرم</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>#FFFDD0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>